<commit_message>
Add customer service type to client import and update customer data
Update documentation and backend logic to include 'TIPO DE ATENDIMENTO' (presential/virtual) during customer data import, and allow for latitude/longitude updates.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 031d314b-746a-4c21-ac74-ddf5bf06e9d4
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/52cb8066-4a28-4875-a42c-7e4d8aae4dad/031d314b-746a-4c21-ac74-ddf5bf06e9d4/P8zbiA3
</commit_message>
<xml_diff>
--- a/attached_assets/modelo_importacao_sales_cards.xlsx
+++ b/attached_assets/modelo_importacao_sales_cards.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Rotas" sheetId="1" r:id="rId1"/>
+    <sheet name="Importação Sales Cards" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:H4"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,80 +422,100 @@
       <c r="D1" t="str">
         <v>FREQUENCIA</v>
       </c>
+      <c r="E1" t="str">
+        <v>LATITUDE</v>
+      </c>
+      <c r="F1" t="str">
+        <v>LONGITUDE</v>
+      </c>
+      <c r="G1" t="str">
+        <v>DATA INICIO</v>
+      </c>
+      <c r="H1" t="str">
+        <v>TIPO DE ATENDIMENTO</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>00.111.222/0001-33</v>
+        <v>00.058.238/0001-78</v>
       </c>
       <c r="B2" t="str">
-        <v>EXEMPLO SUPERMERCADO 1</v>
+        <v>SUPERMERCADO PINTA SILGO</v>
       </c>
       <c r="C2" t="str">
-        <v>SEGUNDA-FEIRA</v>
+        <v>QUARTA-FEIRA</v>
       </c>
       <c r="D2" t="str">
         <v>SEMANAL</v>
+      </c>
+      <c r="E2">
+        <v>-16.6542229</v>
+      </c>
+      <c r="F2">
+        <v>-49.2728202</v>
+      </c>
+      <c r="G2" t="str">
+        <v>25/10/2025</v>
+      </c>
+      <c r="H2" t="str">
+        <v>PRESENCIAL</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>44.555.666/0001-77</v>
+        <v>00.065.979/0001-86</v>
       </c>
       <c r="B3" t="str">
-        <v>EXEMPLO PADARIA 2</v>
+        <v>MERCADINHO JAO</v>
       </c>
       <c r="C3" t="str">
-        <v>TERÇA-FEIRA</v>
+        <v>SEGUNDA-FEIRA</v>
       </c>
       <c r="D3" t="str">
         <v>QUINZENAL</v>
+      </c>
+      <c r="E3">
+        <v>-16.234567</v>
+      </c>
+      <c r="F3">
+        <v>-48.876543</v>
+      </c>
+      <c r="G3" t="str">
+        <v>28/10/2025</v>
+      </c>
+      <c r="H3" t="str">
+        <v>VIRTUAL</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>88.999.000/0001-11</v>
+        <v>00.066.852/0001-81</v>
       </c>
       <c r="B4" t="str">
-        <v>EXEMPLO MERCADINHO 3</v>
+        <v>SUPERMERCADO RIO DAS PEDRAS</v>
       </c>
       <c r="C4" t="str">
-        <v>QUARTA-FEIRA</v>
+        <v>TERÇA-FEIRA</v>
       </c>
       <c r="D4" t="str">
-        <v>SEMANAL</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>12.345.678/0001-99</v>
-      </c>
-      <c r="B5" t="str">
-        <v>EXEMPLO DISTRIBUIDORA 4</v>
-      </c>
-      <c r="C5" t="str">
-        <v>QUINTA-FEIRA</v>
-      </c>
-      <c r="D5" t="str">
         <v>MENSAL</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>98.765.432/0001-00</v>
-      </c>
-      <c r="B6" t="str">
-        <v>EXEMPLO LOJA 5</v>
-      </c>
-      <c r="C6" t="str">
-        <v>SEXTA-FEIRA</v>
-      </c>
-      <c r="D6" t="str">
-        <v>SEMANAL</v>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>01/11/2025</v>
+      </c>
+      <c r="H4" t="str">
+        <v>PRESENCIAL</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>